<commit_message>
screening design notes and alignment
</commit_message>
<xml_diff>
--- a/data/consistency-check-datasets/screening/annotated_screening_dataset.xlsx
+++ b/data/consistency-check-datasets/screening/annotated_screening_dataset.xlsx
@@ -4,11 +4,11 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Readme" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="train-sample" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="l0-sample" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="search-sample" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'train-sample'!$A$1:$I$101</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'l0-sample'!$A$1:$I$101</definedName>
     <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'search-sample'!$A$1:$G$401</definedName>
   </definedNames>
   <calcPr/>
@@ -79,7 +79,7 @@
     <t>Purpose in consistency checking</t>
   </si>
   <si>
-    <t>train-sample</t>
+    <t>l0-sample</t>
   </si>
   <si>
     <r>
@@ -110,14 +110,14 @@
         <b/>
         <color theme="1"/>
       </rPr>
-      <t>from the train split</t>
+      <t>from the screening dataset</t>
     </r>
     <r>
       <rPr>
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t xml:space="preserve"> of the screening dataset was drawn and manually coded after reading titles and abstracts. 
+      <t xml:space="preserve"> was drawn and manually coded after reading titles and abstracts. 
 In their original source, each of these records was adopted from a previously published review, where it had been read in full and marked "Eligible" by the review authors. Here, we re-read the titles and abstracts of these records in line with our eligibility criteria and relabelled them to measure consistency.
 </t>
     </r>
@@ -7695,7 +7695,7 @@
     <mergeCell ref="H11:K11"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink display="train-sample" location="'train-sample'!A1" ref="B10"/>
+    <hyperlink display="l0-sample" location="'l0-sample'!A1" ref="B10"/>
     <hyperlink display="search-sample" location="'search-sample'!A1" ref="B11"/>
   </hyperlinks>
   <drawing r:id="rId1"/>

</xml_diff>